<commit_message>
Make aggregation manifest hashes cross-platform
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/aggregation_v2/validation/DQR_aggregation_validation.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/aggregation_v2/validation/DQR_aggregation_validation.xlsx
@@ -20,7 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pending_registry" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'input_freshness'!$A$1:$H$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'input_freshness'!$A$1:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'contract_checks'!$A$1:$C$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'complete_case_identity'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'aggregator_comparison'!$A$1:$N$9</definedName>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -476,6 +476,7 @@
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,6 +520,11 @@
           <t>sha256_match</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>hash_method</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -555,6 +561,11 @@
       <c r="H2" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -580,17 +591,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>bf56f0bf414e88a625d2be12cd8e7a07e16e4482477c25ebfd25311abc34b743</t>
+          <t>a32bf94f989fc19cbcfc57a1b00e1dff50c742b4b586c51f6750383d9ef24788</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>bf56f0bf414e88a625d2be12cd8e7a07e16e4482477c25ebfd25311abc34b743</t>
+          <t>a32bf94f989fc19cbcfc57a1b00e1dff50c742b4b586c51f6750383d9ef24788</t>
         </is>
       </c>
       <c r="H3" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>sha256_utf8_lf_canonical</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -627,6 +643,11 @@
       <c r="H4" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -652,17 +673,22 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>5cc638b1885e5c3d67742f4e0ad9562b3f1d289cac028fda327350340c93afbc</t>
+          <t>2cbc9dd6ce88ade8e73a7b09acd46a06d39e34b3e1acfdef77529763633cfea9</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>5cc638b1885e5c3d67742f4e0ad9562b3f1d289cac028fda327350340c93afbc</t>
+          <t>2cbc9dd6ce88ade8e73a7b09acd46a06d39e34b3e1acfdef77529763633cfea9</t>
         </is>
       </c>
       <c r="H5" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>sha256_utf8_lf_canonical</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -699,6 +725,11 @@
       <c r="H6" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -724,17 +755,22 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>acba3dd3b937f220337f5fee506f403786565620cda1802a776488e92a228010</t>
+          <t>c15b6316f74f1f165914ed4ba1118c25754301b2cb8ee00fea38126c0e7b41b6</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>acba3dd3b937f220337f5fee506f403786565620cda1802a776488e92a228010</t>
+          <t>c15b6316f74f1f165914ed4ba1118c25754301b2cb8ee00fea38126c0e7b41b6</t>
         </is>
       </c>
       <c r="H7" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>sha256_utf8_lf_canonical</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -771,6 +807,11 @@
       <c r="H8" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -796,17 +837,22 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>8523cf5941017e53d93b313b240347a0737574c18f7746959c1bba963cabb424</t>
+          <t>fff48c27a9245aca07c9f4900f30aa130b576c297e7e6fca6ef1c901e97759e7</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>8523cf5941017e53d93b313b240347a0737574c18f7746959c1bba963cabb424</t>
+          <t>fff48c27a9245aca07c9f4900f30aa130b576c297e7e6fca6ef1c901e97759e7</t>
         </is>
       </c>
       <c r="H9" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>sha256_utf8_lf_canonical</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -843,6 +889,11 @@
       <c r="H10" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -879,6 +930,11 @@
       <c r="H11" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -904,17 +960,22 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>cc813c7f7c8b873cf6ac7ab76015849c4a00591259d3abc2e7bfc494992523fd</t>
+          <t>af675865af284c30f8a44d3b7aacca3a99ed5370eece6b1b5c9bb31ff8bcd79a</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>cc813c7f7c8b873cf6ac7ab76015849c4a00591259d3abc2e7bfc494992523fd</t>
+          <t>af675865af284c30f8a44d3b7aacca3a99ed5370eece6b1b5c9bb31ff8bcd79a</t>
         </is>
       </c>
       <c r="H12" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>sha256_utf8_lf_canonical</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -940,17 +1001,22 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>ec401c6052d3c339e95f508a24baf4b7c5f74f499518bf71e2faebf27c0f79e7</t>
+          <t>8566e80da99727602e35eb127221e9a61c6f781b79cdd42a2f8117c34e5fbf7e</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>ec401c6052d3c339e95f508a24baf4b7c5f74f499518bf71e2faebf27c0f79e7</t>
+          <t>8566e80da99727602e35eb127221e9a61c6f781b79cdd42a2f8117c34e5fbf7e</t>
         </is>
       </c>
       <c r="H13" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>sha256_utf8_lf_canonical</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -987,6 +1053,11 @@
       <c r="H14" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1023,6 +1094,11 @@
       <c r="H15" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1059,6 +1135,11 @@
       <c r="H16" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1095,6 +1176,11 @@
       <c r="H17" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1131,9 +1217,14 @@
       <c r="H18" s="2" t="b">
         <v>1</v>
       </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>sha256_raw_bytes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:I18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>